<commit_message>
feat: daily diary compilation, dynamic form improvements, and record linkage updates
</commit_message>
<xml_diff>
--- a/Master/Sample Case Reg..xlsx
+++ b/Master/Sample Case Reg..xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DPI\FIR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DPI\FIR\pharos-prototype\Master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{78804FC9-8556-4B1A-9A4F-187CE5CB926D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11063707-2F7E-47A4-9C76-F087AC38F357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B484A1A1-A2EC-4440-A4A0-ECC42A4410EE}"/>
   </bookViews>
@@ -34,10 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="161">
-  <si>
-    <t>UID</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="159">
   <si>
     <t>P.S.</t>
   </si>
@@ -120,16 +117,10 @@
     <t>CHARGE SHEET</t>
   </si>
   <si>
-    <t>e-Theft</t>
-  </si>
-  <si>
     <t>Other IPC</t>
   </si>
   <si>
     <t>POLICE INVESTIGATION REPORT(PIR-JCL)</t>
-  </si>
-  <si>
-    <t>e-MVT</t>
   </si>
   <si>
     <t>Other BNS</t>
@@ -518,6 +509,9 @@
   </si>
   <si>
     <t>Unnatural Offences(SODOMY)</t>
+  </si>
+  <si>
+    <t>Unique Case ID</t>
   </si>
 </sst>
 </file>
@@ -667,15 +661,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -688,6 +673,15 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1006,947 +1000,942 @@
   <dimension ref="A1:X120"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="19" max="19" width="35.33203125" customWidth="1"/>
-    <col min="20" max="20" width="58.77734375" customWidth="1"/>
-    <col min="21" max="21" width="75.77734375" customWidth="1"/>
+    <col min="3" max="4" width="14.6640625" customWidth="1"/>
+    <col min="20" max="20" width="35.33203125" customWidth="1"/>
+    <col min="21" max="21" width="58.77734375" customWidth="1"/>
+    <col min="22" max="22" width="75.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="13"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="5"/>
-      <c r="S1" s="6" t="s">
+      <c r="T1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="U1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="V1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="G2" s="5"/>
+      <c r="H2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="8"/>
-      <c r="H2" s="9" t="s">
+      <c r="I2" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="J2" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="O2" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="P2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="O2" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="P2" s="10" t="s">
+      <c r="Q2" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="Q2" s="10" t="s">
+      <c r="R2" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="R2" s="10" t="s">
+      <c r="T2" s="8"/>
+      <c r="U2" s="8"/>
+      <c r="V2" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="S2" s="11"/>
-      <c r="T2" s="11"/>
-      <c r="U2" s="7" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="T3" s="8"/>
+      <c r="U3" s="8"/>
+      <c r="V3" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="S3" s="11"/>
-      <c r="T3" s="11"/>
-      <c r="U3" s="7" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="T4" s="8"/>
+      <c r="U4" s="8"/>
+      <c r="V4" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="F5" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="S4" s="11"/>
-      <c r="T4" s="11"/>
-      <c r="U4" s="7" t="s">
+      <c r="T5" s="8"/>
+      <c r="U5" s="8"/>
+      <c r="V5" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="C5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" s="7" t="s">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="F6" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="S5" s="11"/>
-      <c r="T5" s="11"/>
-      <c r="U5" s="7" t="s">
+      <c r="T6" s="8"/>
+      <c r="U6" s="8"/>
+      <c r="V6" s="4" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="C6" t="s">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="F7" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="T7" s="8"/>
+      <c r="U7" s="8"/>
+      <c r="V7" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="S6" s="11"/>
-      <c r="T6" s="11"/>
-      <c r="U6" s="7" t="s">
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="F8" s="4" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="E7" s="7" t="s">
+      <c r="T8" s="8"/>
+      <c r="U8" s="8"/>
+      <c r="V8" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="S7" s="11"/>
-      <c r="T7" s="11"/>
-      <c r="U7" s="7" t="s">
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="F9" s="4" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="E8" s="7" t="s">
+      <c r="T9" s="8"/>
+      <c r="U9" s="8"/>
+      <c r="V9" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="S8" s="11"/>
-      <c r="T8" s="11"/>
-      <c r="U8" s="7" t="s">
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="F10" s="4" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="E9" s="7" t="s">
+      <c r="T10" s="8"/>
+      <c r="U10" s="8"/>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="F11" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="S9" s="11"/>
-      <c r="T9" s="11"/>
-      <c r="U9" s="7" t="s">
+      <c r="T11" s="8"/>
+      <c r="U11" s="8"/>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="F12" s="4" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="E10" s="7" t="s">
+      <c r="T12" s="8"/>
+      <c r="U12" s="8"/>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="F13" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="S10" s="11"/>
-      <c r="T10" s="11"/>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="E11" s="7" t="s">
+      <c r="T13" s="8"/>
+      <c r="U13" s="8"/>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="F14" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="S11" s="11"/>
-      <c r="T11" s="11"/>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="E12" s="7" t="s">
+      <c r="T14" s="8"/>
+      <c r="U14" s="8"/>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="F15" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="S12" s="11"/>
-      <c r="T12" s="11"/>
-    </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="E13" s="7" t="s">
+      <c r="T15" s="8"/>
+      <c r="U15" s="8"/>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="F16" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="S13" s="11"/>
-      <c r="T13" s="11"/>
-    </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="E14" s="7" t="s">
+      <c r="T16" s="8"/>
+      <c r="U16" s="8"/>
+    </row>
+    <row r="17" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F17" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S14" s="11"/>
-      <c r="T14" s="11"/>
-    </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="E15" s="7" t="s">
+      <c r="T17" s="8"/>
+      <c r="U17" s="8"/>
+    </row>
+    <row r="18" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F18" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="S15" s="11"/>
-      <c r="T15" s="11"/>
-    </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="E16" s="7" t="s">
+      <c r="T18" s="8"/>
+      <c r="U18" s="8"/>
+    </row>
+    <row r="19" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F19" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="S16" s="11"/>
-      <c r="T16" s="11"/>
-    </row>
-    <row r="17" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E17" s="7" t="s">
+      <c r="T19" s="8"/>
+      <c r="U19" s="8"/>
+    </row>
+    <row r="20" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F20" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="S17" s="11"/>
-      <c r="T17" s="11"/>
-    </row>
-    <row r="18" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E18" s="7" t="s">
+      <c r="T20" s="8"/>
+      <c r="U20" s="8"/>
+    </row>
+    <row r="21" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F21" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="S18" s="11"/>
-      <c r="T18" s="11"/>
-    </row>
-    <row r="19" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E19" s="7" t="s">
+      <c r="T21" s="8"/>
+      <c r="U21" s="8"/>
+    </row>
+    <row r="22" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F22" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="S19" s="11"/>
-      <c r="T19" s="11"/>
-    </row>
-    <row r="20" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E20" s="7" t="s">
+      <c r="T22" s="8"/>
+      <c r="U22" s="8"/>
+    </row>
+    <row r="23" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F23" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="S20" s="11"/>
-      <c r="T20" s="11"/>
-    </row>
-    <row r="21" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E21" s="7" t="s">
+      <c r="T23" s="8"/>
+      <c r="U23" s="8"/>
+    </row>
+    <row r="24" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F24" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="S21" s="11"/>
-      <c r="T21" s="11"/>
-    </row>
-    <row r="22" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E22" s="7" t="s">
+      <c r="T24" s="8"/>
+      <c r="U24" s="8"/>
+    </row>
+    <row r="25" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F25" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="S22" s="11"/>
-      <c r="T22" s="11"/>
-    </row>
-    <row r="23" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E23" s="7" t="s">
+      <c r="T25" s="8"/>
+      <c r="U25" s="8"/>
+    </row>
+    <row r="26" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F26" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="S23" s="11"/>
-      <c r="T23" s="11"/>
-    </row>
-    <row r="24" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E24" s="7" t="s">
+      <c r="T26" s="8"/>
+      <c r="U26" s="8"/>
+    </row>
+    <row r="27" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F27" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="S24" s="11"/>
-      <c r="T24" s="11"/>
-    </row>
-    <row r="25" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E25" s="7" t="s">
+      <c r="T27" s="8"/>
+      <c r="U27" s="8"/>
+    </row>
+    <row r="28" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F28" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="S25" s="11"/>
-      <c r="T25" s="11"/>
-    </row>
-    <row r="26" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E26" s="7" t="s">
+      <c r="T28" s="8"/>
+      <c r="U28" s="8"/>
+    </row>
+    <row r="29" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F29" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="S26" s="11"/>
-      <c r="T26" s="11"/>
-    </row>
-    <row r="27" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E27" s="7" t="s">
+      <c r="T29" s="8"/>
+      <c r="U29" s="8"/>
+    </row>
+    <row r="30" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F30" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="S27" s="11"/>
-      <c r="T27" s="11"/>
-    </row>
-    <row r="28" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E28" s="7" t="s">
+      <c r="T30" s="8"/>
+      <c r="U30" s="8"/>
+    </row>
+    <row r="31" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F31" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="S28" s="11"/>
-      <c r="T28" s="11"/>
-    </row>
-    <row r="29" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E29" s="7" t="s">
+      <c r="T31" s="8"/>
+      <c r="U31" s="8"/>
+    </row>
+    <row r="32" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F32" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="S29" s="11"/>
-      <c r="T29" s="11"/>
-    </row>
-    <row r="30" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E30" s="7" t="s">
+      <c r="T32" s="8"/>
+      <c r="U32" s="8"/>
+    </row>
+    <row r="33" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F33" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="S30" s="11"/>
-      <c r="T30" s="11"/>
-    </row>
-    <row r="31" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E31" s="7" t="s">
+      <c r="T33" s="8"/>
+      <c r="U33" s="8"/>
+    </row>
+    <row r="34" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F34" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="S31" s="11"/>
-      <c r="T31" s="11"/>
-    </row>
-    <row r="32" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E32" s="7" t="s">
+      <c r="T34" s="8"/>
+      <c r="U34" s="8"/>
+    </row>
+    <row r="35" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F35" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="S32" s="11"/>
-      <c r="T32" s="11"/>
-    </row>
-    <row r="33" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E33" s="7" t="s">
+      <c r="G35" s="10"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="10"/>
+      <c r="J35" s="10"/>
+      <c r="K35" s="10"/>
+      <c r="L35" s="10"/>
+      <c r="M35" s="10"/>
+      <c r="N35" s="10"/>
+      <c r="O35" s="10"/>
+      <c r="P35" s="10"/>
+      <c r="Q35" s="10"/>
+      <c r="R35" s="10"/>
+      <c r="S35" s="10"/>
+      <c r="T35" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="S33" s="11"/>
-      <c r="T33" s="11"/>
-    </row>
-    <row r="34" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E34" s="7" t="s">
+      <c r="U35" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="S34" s="11"/>
-      <c r="T34" s="11"/>
-    </row>
-    <row r="35" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E35" s="12" t="s">
+    </row>
+    <row r="36" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F36" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="13"/>
-      <c r="J35" s="13"/>
-      <c r="K35" s="13"/>
-      <c r="L35" s="13"/>
-      <c r="M35" s="13"/>
-      <c r="N35" s="13"/>
-      <c r="O35" s="13"/>
-      <c r="P35" s="13"/>
-      <c r="Q35" s="13"/>
-      <c r="R35" s="13"/>
-      <c r="S35" s="13" t="s">
+      <c r="T36" s="8"/>
+      <c r="U36" s="8"/>
+    </row>
+    <row r="37" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F37" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="T35" s="13" t="s">
+      <c r="T37" s="8"/>
+      <c r="U37" s="8"/>
+    </row>
+    <row r="38" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F38" s="4" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="36" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E36" s="7" t="s">
+      <c r="T38" s="8"/>
+      <c r="U38" s="8"/>
+    </row>
+    <row r="39" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F39" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="S36" s="11"/>
-      <c r="T36" s="11"/>
-    </row>
-    <row r="37" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E37" s="7" t="s">
+      <c r="T39" s="8"/>
+      <c r="U39" s="8"/>
+    </row>
+    <row r="40" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F40" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="S37" s="11"/>
-      <c r="T37" s="11"/>
-    </row>
-    <row r="38" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E38" s="7" t="s">
+      <c r="T40" s="8"/>
+      <c r="U40" s="8"/>
+    </row>
+    <row r="41" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F41" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="S38" s="11"/>
-      <c r="T38" s="11"/>
-    </row>
-    <row r="39" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E39" s="7" t="s">
+      <c r="T41" s="8"/>
+      <c r="U41" s="8"/>
+    </row>
+    <row r="42" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F42" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="S39" s="11"/>
-      <c r="T39" s="11"/>
-    </row>
-    <row r="40" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E40" s="7" t="s">
+      <c r="T42" s="8"/>
+      <c r="U42" s="8"/>
+    </row>
+    <row r="43" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F43" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="S40" s="11"/>
-      <c r="T40" s="11"/>
-    </row>
-    <row r="41" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E41" s="7" t="s">
+      <c r="T43" s="8"/>
+      <c r="U43" s="8"/>
+    </row>
+    <row r="44" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F44" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="S41" s="11"/>
-      <c r="T41" s="11"/>
-    </row>
-    <row r="42" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E42" s="7" t="s">
+      <c r="T44" s="8"/>
+      <c r="U44" s="8"/>
+    </row>
+    <row r="45" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F45" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="S42" s="11"/>
-      <c r="T42" s="11"/>
-    </row>
-    <row r="43" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E43" s="7" t="s">
+      <c r="T45" s="8"/>
+      <c r="U45" s="8"/>
+    </row>
+    <row r="46" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F46" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="S43" s="11"/>
-      <c r="T43" s="11"/>
-    </row>
-    <row r="44" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E44" s="7" t="s">
+      <c r="T46" s="8"/>
+      <c r="U46" s="8"/>
+    </row>
+    <row r="47" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F47" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="S44" s="11"/>
-      <c r="T44" s="11"/>
-    </row>
-    <row r="45" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E45" s="7" t="s">
+      <c r="T47" s="8"/>
+      <c r="U47" s="8"/>
+    </row>
+    <row r="48" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F48" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="S45" s="11"/>
-      <c r="T45" s="11"/>
-    </row>
-    <row r="46" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E46" s="7" t="s">
+      <c r="T48" s="8"/>
+      <c r="U48" s="8"/>
+    </row>
+    <row r="49" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F49" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="S46" s="11"/>
-      <c r="T46" s="11"/>
-    </row>
-    <row r="47" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E47" s="7" t="s">
+      <c r="T49" s="8"/>
+      <c r="U49" s="8"/>
+    </row>
+    <row r="50" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F50" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="S47" s="11"/>
-      <c r="T47" s="11"/>
-    </row>
-    <row r="48" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E48" s="7" t="s">
+      <c r="T50" s="8"/>
+      <c r="U50" s="8"/>
+    </row>
+    <row r="51" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F51" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="S48" s="11"/>
-      <c r="T48" s="11"/>
-    </row>
-    <row r="49" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E49" s="7" t="s">
+      <c r="T51" s="8"/>
+      <c r="U51" s="8"/>
+    </row>
+    <row r="52" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F52" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="S49" s="11"/>
-      <c r="T49" s="11"/>
-    </row>
-    <row r="50" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E50" s="7" t="s">
+      <c r="T52" s="8"/>
+      <c r="U52" s="8"/>
+    </row>
+    <row r="53" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F53" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="S50" s="11"/>
-      <c r="T50" s="11"/>
-    </row>
-    <row r="51" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E51" s="7" t="s">
+      <c r="T53" s="8"/>
+      <c r="U53" s="8"/>
+    </row>
+    <row r="54" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F54" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="S51" s="11"/>
-      <c r="T51" s="11"/>
-    </row>
-    <row r="52" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E52" s="7" t="s">
+      <c r="T54" s="8"/>
+      <c r="U54" s="8"/>
+    </row>
+    <row r="55" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F55" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="S52" s="11"/>
-      <c r="T52" s="11"/>
-    </row>
-    <row r="53" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E53" s="7" t="s">
+      <c r="T55" s="8"/>
+      <c r="U55" s="8"/>
+    </row>
+    <row r="56" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F56" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="S53" s="11"/>
-      <c r="T53" s="11"/>
-    </row>
-    <row r="54" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E54" s="7" t="s">
+      <c r="T56" s="8"/>
+      <c r="U56" s="8"/>
+    </row>
+    <row r="57" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F57" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="S54" s="11"/>
-      <c r="T54" s="11"/>
-    </row>
-    <row r="55" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E55" s="7" t="s">
+      <c r="T57" s="8"/>
+      <c r="U57" s="8"/>
+    </row>
+    <row r="58" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F58" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="S55" s="11"/>
-      <c r="T55" s="11"/>
-    </row>
-    <row r="56" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E56" s="7" t="s">
+      <c r="T58" s="8"/>
+      <c r="U58" s="8"/>
+    </row>
+    <row r="59" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F59" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="S56" s="11"/>
-      <c r="T56" s="11"/>
-    </row>
-    <row r="57" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E57" s="7" t="s">
+      <c r="T59" s="8"/>
+      <c r="U59" s="8"/>
+    </row>
+    <row r="60" spans="6:21" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="F60" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="S57" s="11"/>
-      <c r="T57" s="11"/>
-    </row>
-    <row r="58" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E58" s="7" t="s">
+      <c r="T60" s="8"/>
+      <c r="U60" s="8"/>
+    </row>
+    <row r="61" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F61" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="S58" s="11"/>
-      <c r="T58" s="11"/>
-    </row>
-    <row r="59" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E59" s="7" t="s">
+      <c r="T61" s="8"/>
+      <c r="U61" s="8"/>
+    </row>
+    <row r="62" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F62" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="S59" s="11"/>
-      <c r="T59" s="11"/>
-    </row>
-    <row r="60" spans="5:20" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="E60" s="14" t="s">
+      <c r="T62" s="8"/>
+      <c r="U62" s="8"/>
+    </row>
+    <row r="63" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F63" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="S60" s="11"/>
-      <c r="T60" s="11"/>
-    </row>
-    <row r="61" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E61" s="7" t="s">
+      <c r="T63" s="8"/>
+      <c r="U63" s="8"/>
+    </row>
+    <row r="64" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F64" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="S61" s="11"/>
-      <c r="T61" s="11"/>
-    </row>
-    <row r="62" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E62" s="7" t="s">
+      <c r="T64" s="8"/>
+      <c r="U64" s="8"/>
+    </row>
+    <row r="65" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F65" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="S62" s="11"/>
-      <c r="T62" s="11"/>
-    </row>
-    <row r="63" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E63" s="7" t="s">
+      <c r="T65" s="8"/>
+      <c r="U65" s="8"/>
+    </row>
+    <row r="66" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F66" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="S63" s="11"/>
-      <c r="T63" s="11"/>
-    </row>
-    <row r="64" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E64" s="7" t="s">
+      <c r="T66" s="8"/>
+      <c r="U66" s="8"/>
+    </row>
+    <row r="67" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F67" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="S64" s="11"/>
-      <c r="T64" s="11"/>
-    </row>
-    <row r="65" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E65" s="7" t="s">
+      <c r="T67" s="8"/>
+      <c r="U67" s="8"/>
+    </row>
+    <row r="68" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F68" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="S65" s="11"/>
-      <c r="T65" s="11"/>
-    </row>
-    <row r="66" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E66" s="7" t="s">
+      <c r="T68" s="8"/>
+      <c r="U68" s="8"/>
+    </row>
+    <row r="69" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F69" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="S66" s="11"/>
-      <c r="T66" s="11"/>
-    </row>
-    <row r="67" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E67" s="7" t="s">
+      <c r="T69" s="8"/>
+      <c r="U69" s="8"/>
+    </row>
+    <row r="70" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F70" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="S67" s="11"/>
-      <c r="T67" s="11"/>
-    </row>
-    <row r="68" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E68" s="7" t="s">
+      <c r="T70" s="8"/>
+      <c r="U70" s="8"/>
+    </row>
+    <row r="71" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F71" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="S68" s="11"/>
-      <c r="T68" s="11"/>
-    </row>
-    <row r="69" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E69" s="7" t="s">
+      <c r="T71" s="8"/>
+      <c r="U71" s="8"/>
+    </row>
+    <row r="72" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F72" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="S69" s="11"/>
-      <c r="T69" s="11"/>
-    </row>
-    <row r="70" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E70" s="7" t="s">
+      <c r="T72" s="8"/>
+      <c r="U72" s="8"/>
+    </row>
+    <row r="73" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F73" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="S70" s="11"/>
-      <c r="T70" s="11"/>
-    </row>
-    <row r="71" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E71" s="7" t="s">
+      <c r="T73" s="8"/>
+      <c r="U73" s="8"/>
+    </row>
+    <row r="74" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F74" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="S71" s="11"/>
-      <c r="T71" s="11"/>
-    </row>
-    <row r="72" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E72" s="7" t="s">
+      <c r="T74" s="8"/>
+      <c r="U74" s="8"/>
+    </row>
+    <row r="75" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F75" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="S72" s="11"/>
-      <c r="T72" s="11"/>
-    </row>
-    <row r="73" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E73" s="7" t="s">
+      <c r="T75" s="8"/>
+      <c r="U75" s="8"/>
+    </row>
+    <row r="76" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F76" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="S73" s="11"/>
-      <c r="T73" s="11"/>
-    </row>
-    <row r="74" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E74" s="7" t="s">
+      <c r="T76" s="8"/>
+      <c r="U76" s="8"/>
+    </row>
+    <row r="77" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F77" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="S74" s="11"/>
-      <c r="T74" s="11"/>
-    </row>
-    <row r="75" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E75" s="7" t="s">
+      <c r="T77" s="8"/>
+      <c r="U77" s="8"/>
+    </row>
+    <row r="78" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F78" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="S75" s="11"/>
-      <c r="T75" s="11"/>
-    </row>
-    <row r="76" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E76" s="7" t="s">
+      <c r="T78" s="8"/>
+      <c r="U78" s="8"/>
+    </row>
+    <row r="79" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F79" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="S76" s="11"/>
-      <c r="T76" s="11"/>
-    </row>
-    <row r="77" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E77" s="7" t="s">
+      <c r="T79" s="8"/>
+      <c r="U79" s="8"/>
+    </row>
+    <row r="80" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F80" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="S77" s="11"/>
-      <c r="T77" s="11"/>
-    </row>
-    <row r="78" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E78" s="7" t="s">
+      <c r="T80" s="8"/>
+      <c r="U80" s="8"/>
+    </row>
+    <row r="81" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F81" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="S78" s="11"/>
-      <c r="T78" s="11"/>
-    </row>
-    <row r="79" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E79" s="7" t="s">
+      <c r="T81" s="8"/>
+      <c r="U81" s="8"/>
+    </row>
+    <row r="82" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F82" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="S79" s="11"/>
-      <c r="T79" s="11"/>
-    </row>
-    <row r="80" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E80" s="7" t="s">
+      <c r="T82" s="8"/>
+      <c r="U82" s="8"/>
+    </row>
+    <row r="83" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F83" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="S80" s="11"/>
-      <c r="T80" s="11"/>
-    </row>
-    <row r="81" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E81" s="7" t="s">
+      <c r="T83" s="8"/>
+      <c r="U83" s="8"/>
+    </row>
+    <row r="84" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F84" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="S81" s="11"/>
-      <c r="T81" s="11"/>
-    </row>
-    <row r="82" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E82" s="7" t="s">
+      <c r="T84" s="8"/>
+      <c r="U84" s="8"/>
+    </row>
+    <row r="85" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F85" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="S82" s="11"/>
-      <c r="T82" s="11"/>
-    </row>
-    <row r="83" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E83" s="7" t="s">
+      <c r="T85" s="8"/>
+      <c r="U85" s="8"/>
+    </row>
+    <row r="86" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F86" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="S83" s="11"/>
-      <c r="T83" s="11"/>
-    </row>
-    <row r="84" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E84" s="7" t="s">
+      <c r="T86" s="8"/>
+      <c r="U86" s="8"/>
+    </row>
+    <row r="87" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F87" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="S84" s="11"/>
-      <c r="T84" s="11"/>
-    </row>
-    <row r="85" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E85" s="7" t="s">
+      <c r="T87" s="8"/>
+      <c r="U87" s="8"/>
+    </row>
+    <row r="88" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F88" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="S85" s="11"/>
-      <c r="T85" s="11"/>
-    </row>
-    <row r="86" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E86" s="7" t="s">
+      <c r="T88" s="8"/>
+      <c r="U88" s="8"/>
+    </row>
+    <row r="89" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F89" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="S86" s="11"/>
-      <c r="T86" s="11"/>
-    </row>
-    <row r="87" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E87" s="7" t="s">
+      <c r="T89" s="8"/>
+      <c r="U89" s="8"/>
+    </row>
+    <row r="90" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F90" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="S87" s="11"/>
-      <c r="T87" s="11"/>
-    </row>
-    <row r="88" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E88" s="7" t="s">
+      <c r="T90" s="8"/>
+      <c r="U90" s="8"/>
+    </row>
+    <row r="91" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F91" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="S88" s="11"/>
-      <c r="T88" s="11"/>
-    </row>
-    <row r="89" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E89" s="7" t="s">
+      <c r="T91" s="8"/>
+      <c r="U91" s="8"/>
+    </row>
+    <row r="92" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F92" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="S89" s="11"/>
-      <c r="T89" s="11"/>
-    </row>
-    <row r="90" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E90" s="7" t="s">
+      <c r="T92" s="8"/>
+      <c r="U92" s="8"/>
+    </row>
+    <row r="93" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F93" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="S90" s="11"/>
-      <c r="T90" s="11"/>
-    </row>
-    <row r="91" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E91" s="7" t="s">
+      <c r="G93" s="10"/>
+      <c r="H93" s="10"/>
+      <c r="I93" s="10"/>
+      <c r="J93" s="10"/>
+      <c r="K93" s="10"/>
+      <c r="L93" s="10"/>
+      <c r="M93" s="10"/>
+      <c r="N93" s="10"/>
+      <c r="O93" s="10"/>
+      <c r="P93" s="10"/>
+      <c r="Q93" s="10"/>
+      <c r="R93" s="10"/>
+      <c r="S93" s="10"/>
+      <c r="T93" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="S91" s="11"/>
-      <c r="T91" s="11"/>
-    </row>
-    <row r="92" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E92" s="7" t="s">
+      <c r="U93" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="S92" s="11"/>
-      <c r="T92" s="11"/>
-    </row>
-    <row r="93" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E93" s="12" t="s">
+    </row>
+    <row r="94" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F94" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="F93" s="13"/>
-      <c r="G93" s="13"/>
-      <c r="H93" s="13"/>
-      <c r="I93" s="13"/>
-      <c r="J93" s="13"/>
-      <c r="K93" s="13"/>
-      <c r="L93" s="13"/>
-      <c r="M93" s="13"/>
-      <c r="N93" s="13"/>
-      <c r="O93" s="13"/>
-      <c r="P93" s="13"/>
-      <c r="Q93" s="13"/>
-      <c r="R93" s="13"/>
-      <c r="S93" s="13" t="s">
+    </row>
+    <row r="95" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F95" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="T93" s="13" t="s">
+    </row>
+    <row r="96" spans="6:21" x14ac:dyDescent="0.3">
+      <c r="F96" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="94" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E94" s="7" t="s">
+    <row r="97" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F97" s="4" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="95" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E95" s="7" t="s">
+    <row r="98" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F98" s="4" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="96" spans="5:20" x14ac:dyDescent="0.3">
-      <c r="E96" s="7" t="s">
+    <row r="99" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F99" s="4" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="97" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E97" s="7" t="s">
+    <row r="100" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F100" s="4" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="98" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E98" s="7" t="s">
+    <row r="101" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F101" s="4" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="99" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E99" s="7" t="s">
+    <row r="102" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F102" s="4" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="100" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E100" s="7" t="s">
+    <row r="103" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F103" s="4" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="101" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E101" s="7" t="s">
+    <row r="104" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F104" s="4" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="102" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E102" s="7" t="s">
+    <row r="105" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F105" s="4" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="103" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E103" s="7" t="s">
+    <row r="106" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F106" s="4" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="104" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E104" s="7" t="s">
+    <row r="107" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F107" s="4" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="105" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E105" s="7" t="s">
+    <row r="108" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F108" s="4" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="106" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E106" s="7" t="s">
+    <row r="109" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F109" s="4" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="107" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E107" s="7" t="s">
+    <row r="110" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F110" s="4" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="108" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E108" s="7" t="s">
+    <row r="111" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F111" s="4" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="109" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E109" s="7" t="s">
+    <row r="112" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F112" s="4" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="110" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E110" s="7" t="s">
+    <row r="113" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F113" s="4" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="111" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E111" s="7" t="s">
+    <row r="114" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F114" s="4" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="112" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E112" s="7" t="s">
+    <row r="115" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F115" s="4" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="113" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E113" s="7" t="s">
+    <row r="116" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F116" s="4" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="114" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E114" s="7" t="s">
+    <row r="117" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F117" s="4" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="115" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E115" s="7" t="s">
+    <row r="118" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F118" s="4" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="116" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E116" s="7" t="s">
+    <row r="119" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F119" s="4" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="117" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E117" s="7" t="s">
+    <row r="120" spans="6:6" x14ac:dyDescent="0.3">
+      <c r="F120" s="4" t="s">
         <v>157</v>
-      </c>
-    </row>
-    <row r="118" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E118" s="7" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="119" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E119" s="7" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="120" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E120" s="7" t="s">
-        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>